<commit_message>
Add Indic LLM pre-training tech report and link it from news
- Add "Scaling Synthetic Pre-training Data and Evaluation for Indic LLMs"
  (arXiv:2610.26006) to publications
- Point the 17 Oct 2026 news item's [tech_report] link to arXiv

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/my_publications.xlsx
+++ b/scripts/my_publications.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$J$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$J$99</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J98"/>
+  <dimension ref="A1:J99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="4" min="1" max="1"/>
@@ -566,32 +566,32 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>NLP/Translation/Evaluation/Indic</t>
+          <t>NLP/LM/Evaluation/Multilingual/Indic</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>IndicQE-APE: A Consolidated Benchmark for Quality Estimation and Automatic Post-Editing for Indic Languages</t>
+          <t>Scaling Synthetic Pre-training Data and Evaluation for Indic LLMs</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>WMT 2026 (to appear)</t>
+          <t>arXiv preprint arXiv:2610.26006</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Diptesh Kanojia, Archchana Sindhujan, Sourabh Deoghare, Daria Sokova, Shenbin Qian, Girish Koushik, Tharindu Ranasinghe, Constantin Orăsan, Chrysoula Zerva, Ricardo Rei, Frédéric Blain, André F. T. Martins, Marco Turchi, Matteo Negri, Anoop Kunchukuttan, Mitesh M. Khapra, Pushpak Bhattacharyya</t>
+          <t>Abhinav Khattar, Aishwarya Chhabra, Ameya Velingker, Anusha Kamath, Brandon Norick, Kanishk Singla, Kiran Praveen, Markus Kliegl, Mohammad Qazim Bhat, Mostofa Patwary, Niket Agarwal, Rajpreet Thethy, Ramani Akkati, Raviraj Joshi, Sai Nishanth Padala, Shuoyang Ding, Sriharsha Niverty, Utkarsh Vaidya, Vitaly Lavrukhin, Yev Meyer, Anoop Kunchukuttan, Mitesh Khapra, Mohammed Safi Ur Rahman Khan, Rudra Murthy, Sumanth Doddapaneni, Thanmay Jayakumar, Ujjwal Sharma</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2608.16344</t>
+          <t>https://arxiv.org/abs/2610.26006</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Pre-print</t>
         </is>
       </c>
       <c r="H2" s="2" t="n"/>
@@ -604,27 +604,27 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>NLP/LM/Evaluation/Multilingual/Indic</t>
+          <t>NLP/Translation/Evaluation/Indic</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>IndicIFEval: A Benchmark for Verifiable Instruction-Following Evaluation in 14 Indic Languages</t>
+          <t>IndicQE-APE: A Consolidated Benchmark for Quality Estimation and Automatic Post-Editing for Indic Languages</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>AACL-IJCNLP 2026 (to appear)</t>
+          <t>WMT 2026 (to appear)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Thanmay Jayakumar, Mohammed Safi Ur Rahman Khan, Raj Dabre, Ratish Puduppully, Anoop Kunchukuttan</t>
+          <t>Diptesh Kanojia, Archchana Sindhujan, Sourabh Deoghare, Daria Sokova, Shenbin Qian, Girish Koushik, Tharindu Ranasinghe, Constantin Orăsan, Chrysoula Zerva, Ricardo Rei, Frédéric Blain, André F. T. Martins, Marco Turchi, Matteo Negri, Anoop Kunchukuttan, Mitesh M. Khapra, Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2602.22125</t>
+          <t>https://arxiv.org/abs/2608.16344</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -642,32 +642,32 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>NLP/Reasoning</t>
+          <t>NLP/LM/Evaluation/Multilingual/Indic</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>RiddleBench: A New Generative Reasoning Benchmark for LLMs</t>
+          <t>IndicIFEval: A Benchmark for Verifiable Instruction-Following Evaluation in 14 Indic Languages</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>EACL 2026 Findings (to appear)</t>
+          <t>AACL-IJCNLP 2026 (to appear)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deepon Halder, Alan Saji, Thanmay Jayakumar, Ratish Puduppully, Anoop Kunchukuttan, Raj Dabre </t>
+          <t>Thanmay Jayakumar, Mohammed Safi Ur Rahman Khan, Raj Dabre, Ratish Puduppully, Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2510.24932</t>
+          <t>https://arxiv.org/abs/2602.22125</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Short Paper</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H4" s="2" t="n"/>
@@ -680,27 +680,27 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>NLP/Reasoning/Multilingual</t>
+          <t>NLP/Reasoning</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>The Reasoning Lingua Franca: A Double-Edged Sword for Multilingual AI</t>
+          <t>RiddleBench: A New Generative Reasoning Benchmark for LLMs</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>EACL 2026 (to appear)</t>
+          <t>EACL 2026 Findings (to appear)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Alan Saji, Raj Dabre, Anoop Kunchukuttan, Ratish Puduppully</t>
+          <t xml:space="preserve">Deepon Halder, Alan Saji, Thanmay Jayakumar, Ratish Puduppully, Anoop Kunchukuttan, Raj Dabre </t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2510.20647</t>
+          <t>https://arxiv.org/abs/2510.24932</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -708,124 +708,124 @@
           <t>Short Paper</t>
         </is>
       </c>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="8" t="n"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>NLP/Reasoning/Multilingual</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>The Reasoning Lingua Franca: A Double-Edged Sword for Multilingual AI</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>EACL 2026 (to appear)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Alan Saji, Raj Dabre, Anoop Kunchukuttan, Ratish Puduppully</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2510.20647</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Short Paper</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>NLP/Translation/Multilingual/Indic</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Pralekha: Cross-lingual Document Alignment for Indic Languages</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>AACL</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Suryanarayanan, Sanjay; Song, Haiyue; Khan, Mohammed Safi Ur Rahman; Kunchukuttan, Anoop; Khapra, Mitesh M; Dabre, Raj; </t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2411.19096</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Full Paper</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>NLP/LM/Multilingual</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>A primer on pretrained multilingual language models</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>ACM Computing Surveys</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Sumanth Doddapaneni,  Gowtham Ramesh,  Mitesh M Khapra,  Anoop Kunchukuttan,  Pratyush Kumar</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://dl.acm.org/doi/abs/10.1145/3727339</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Survey</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>jnoUuGcAAAAJ:z_wVstp3MssC</t>
         </is>
       </c>
-      <c r="J7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>NLP/Multilingual/Indic</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>IndicRAGSuite: Large-Scale Datasets and a Benchmark for Indian Language RAG Systems</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>arXiv preprint arXiv:2506.01615</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Pasunuti Prasanjith, Prathmesh B More, Anoop Kunchukuttan, Raj Dabre</t>
-        </is>
-      </c>
-      <c r="F8" s="11" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2506.01615</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Pre-print</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="8" t="n"/>
+      <c r="J8" s="7" t="n"/>
     </row>
     <row r="9" ht="75" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -833,32 +833,32 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>NLP/LM/Multilingual</t>
+          <t>NLP/Multilingual/Indic</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>Data and Model Centric Approaches for Expansion of Large Language Models to New languages</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EMNLP </t>
+          <t>IndicRAGSuite: Large-Scale Datasets and a Benchmark for Indian Language RAG Systems</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>arXiv preprint arXiv:2506.01615</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan, Raj Dabre, Rudramurthy V, Mohammed Safi Ur Rahman, Thanmay Jayakumar</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>https://github.com/anoopkunchukuttan/multilingual_extend_llm</t>
+          <t>Pasunuti Prasanjith, Prathmesh B More, Anoop Kunchukuttan, Raj Dabre</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2506.01615</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Tutorial</t>
+          <t>Pre-print</t>
         </is>
       </c>
       <c r="H9" s="2" t="n"/>
@@ -874,33 +874,34 @@
           <t>NLP/LM/Multilingual</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>RomanLens: The Role Of Latent Romanization In Multilinguality In LLMs</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ACL 2025 Findings </t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Alan Saji, Jaavid Aktar Husain, Thanmay Jayakumar, Raj Dabre, Anoop Kunchukuttan, Ratish Puduppully</t>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Data and Model Centric Approaches for Expansion of Large Language Models to New languages</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EMNLP </t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Anoop Kunchukuttan, Raj Dabre, Rudramurthy V, Mohammed Safi Ur Rahman, Thanmay Jayakumar</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2502.07424</t>
+          <t>https://github.com/anoopkunchukuttan/multilingual_extend_llm</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
+      <c r="J10" s="8" t="n"/>
     </row>
     <row r="11" ht="75" customHeight="1">
       <c r="A11" s="3" t="n">
@@ -908,27 +909,27 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>NLP/Speech/Translation/Indic/Multilingual/Multimodal</t>
+          <t>NLP/LM/Multilingual</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>BhasaAnuvaad: A Speech Translation Dataset for 13 Indian Languages</t>
+          <t>RomanLens: The Role Of Latent Romanization In Multilinguality In LLMs</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>ACL 2025</t>
+          <t xml:space="preserve">ACL 2025 Findings </t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jain, Sparsh; Sankar, Ashwin; Choudhary, Devilal; Suman, Dhairya; Narasimhan, Nikhil; Khan, Mohammed Safi Ur Rahman; Kunchukuttan, Anoop; Khapra, Mitesh M; Dabre, Raj; </t>
+          <t>Alan Saji, Jaavid Aktar Husain, Thanmay Jayakumar, Raj Dabre, Anoop Kunchukuttan, Ratish Puduppully</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2411.04699</t>
+          <t>https://arxiv.org/abs/2502.07424</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,17 +941,17 @@
       <c r="I11" s="2" t="n"/>
     </row>
     <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="3" t="n">
         <v>2025</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>NLP/LM/Evaluation/Multilingual</t>
+          <t>NLP/Speech/Translation/Indic/Multilingual/Multimodal</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Cross-Lingual Auto Evaluation for Assessing Multilingual LLMs</t>
+          <t>BhasaAnuvaad: A Speech Translation Dataset for 13 Indian Languages</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -960,12 +961,12 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doddapaneni, Sumanth; Khan, Mohammed Safi Ur Rahman; Venkatesh, Dilip; Dabre, Raj; Kunchukuttan, Anoop; Khapra, Mitesh M; </t>
+          <t xml:space="preserve">Jain, Sparsh; Sankar, Ashwin; Choudhary, Devilal; Suman, Dhairya; Narasimhan, Nikhil; Khan, Mohammed Safi Ur Rahman; Kunchukuttan, Anoop; Khapra, Mitesh M; Dabre, Raj; </t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2410.13394</t>
+          <t>https://arxiv.org/abs/2411.04699</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -978,73 +979,73 @@
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>NLP/LM/Indic</t>
+        <v>2025</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>NLP/LM/Evaluation/Multilingual</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Airavata: Introducing Hindi Instruction-tuned LLM</t>
+          <t>Cross-Lingual Auto Evaluation for Assessing Multilingual LLMs</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>arXiv preprint arXiv:2401.15006</t>
+          <t>ACL 2025</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Jay Gala, Thanmay Jayakumar, Jaavid Aktar Husain, Aswanth Kumar M, Mohammed Safi Ur Rahman Khan, Diptesh Kanojia, Ratish Puduppully, Mitesh M. Khapra, Raj Dabre, Rudra Murthy, Anoop Kunchukuttan</t>
+          <t xml:space="preserve">Doddapaneni, Sumanth; Khan, Mohammed Safi Ur Rahman; Venkatesh, Dilip; Dabre, Raj; Kunchukuttan, Anoop; Khapra, Mitesh M; </t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2401.15006</t>
+          <t>https://arxiv.org/abs/2410.13394</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Pre-print</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
     </row>
     <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="4" t="n">
         <v>2024</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>NLP/LM/Multilingual</t>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>NLP/LM/Indic</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Extending English Large Language Models to New Languages: A Survey</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Anoop Kunchukuttan</t>
+          <t>Airavata: Introducing Hindi Instruction-tuned LLM</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>arXiv preprint arXiv:2401.15006</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Jay Gala, Thanmay Jayakumar, Jaavid Aktar Husain, Aswanth Kumar M, Mohammed Safi Ur Rahman Khan, Diptesh Kanojia, Ratish Puduppully, Mitesh M. Khapra, Raj Dabre, Rudra Murthy, Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://github.com/anoopkunchukuttan/multilingual_extend_llm</t>
+          <t>https://arxiv.org/abs/2401.15006</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Tutorial</t>
+          <t>Pre-print</t>
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
@@ -1054,34 +1055,34 @@
       <c r="A15" s="3" t="n">
         <v>2024</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>NLP/Multilingual</t>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>NLP/LM/Multilingual</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Synthetic Data Generation and Joint Learning for Robust Code-Mixed Translation</t>
+          <t>Extending English Large Language Models to New Languages: A Survey</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>COLING-LREC</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kartik; Soni, Sanjana; Kunchukuttan, Anoop; Chakraborty, Tanmoy; Akhtar, Md. Shad; </t>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2024.lrec-main.1345/</t>
+          <t>https://github.com/anoopkunchukuttan/multilingual_extend_llm</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="H15" s="2" t="n"/>
@@ -1093,27 +1094,27 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>NLP/LM</t>
+          <t>NLP/Multilingual</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>An Empirical Comparison of Vocabulary Expansion and Initialization Approaches for Language Models</t>
+          <t>Synthetic Data Generation and Joint Learning for Robust Code-Mixed Translation</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>CoNLL</t>
+          <t>COLING-LREC</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mundra, Nandini; Kishore, Aditya Nanda; Dabre, Raj; Puduppully, Ratish; Kunchukuttan, Anoop; Khapra, Mitesh M; </t>
+          <t xml:space="preserve">Kartik; Soni, Sanjana; Kunchukuttan, Anoop; Chakraborty, Tanmoy; Akhtar, Md. Shad; </t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2024.conll-1.8/</t>
+          <t>https://aclanthology.org/2024.lrec-main.1345/</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1125,44 +1126,41 @@
       <c r="I16" s="2" t="n"/>
     </row>
     <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="3" t="n">
         <v>2024</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>NLP/LM/Indic/Multilingual</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>IndicLLMSuite: A Blueprint for Creating Pre-training and Fine-Tuning Datasets for Indian Languages.</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>ACL</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Khan, Mohammed Safi Ur Rahman, Priyam Mehta, Ananth Sankar, Umashankar Kumaravelan, Sumanth Doddapaneni, Sparsh Jain, Anoop Kunchukuttan, Pratyush Kumar, Raj Dabre, and Mitesh M. Khapra</t>
+          <t>NLP/LM</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>An Empirical Comparison of Vocabulary Expansion and Initialization Approaches for Language Models</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>CoNLL</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mundra, Nandini; Kishore, Aditya Nanda; Dabre, Raj; Puduppully, Ratish; Kunchukuttan, Anoop; Khapra, Mitesh M; </t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2024.acl-long.843/</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
+          <t>https://aclanthology.org/2024.conll-1.8/</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Full Paper</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>Oustanding Paper Award</t>
-        </is>
-      </c>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="4" t="n">
@@ -1170,12 +1168,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>NLP/LM/Multilingual</t>
+          <t>NLP/LM/Indic/Multilingual</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>RomanSetu: Efficiently unlocking multilingual capabilities of Large Language Models models via Romanization.</t>
+          <t>IndicLLMSuite: A Blueprint for Creating Pre-training and Fine-Tuning Datasets for Indian Languages.</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1185,12 +1183,12 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Husain, Jaavid Aktar, Raj Dabre, Aswanth Kumar, Ratish Puduppully, and Anoop Kunchukuttan</t>
+          <t>Khan, Mohammed Safi Ur Rahman, Priyam Mehta, Ananth Sankar, Umashankar Kumaravelan, Sumanth Doddapaneni, Sparsh Jain, Anoop Kunchukuttan, Pratyush Kumar, Raj Dabre, and Mitesh M. Khapra</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2024.acl-long.833</t>
+          <t>https://aclanthology.org/2024.acl-long.843/</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1200,7 +1198,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Area Chair Award</t>
+          <t>Oustanding Paper Award</t>
         </is>
       </c>
     </row>
@@ -1210,12 +1208,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Evaluation/Indic</t>
+          <t>NLP/LM/Multilingual</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>How Good is Zero-Shot MT Evaluation for Low Resource Indian Languages</t>
+          <t>RomanSetu: Efficiently unlocking multilingual capabilities of Large Language Models models via Romanization.</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1225,17 +1223,22 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Anushka Singh, Ananya B. Sai, Raj Dabre, Ratish Puduppully, Anoop Kunchukuttan, Mitesh M Khapra</t>
+          <t>Husain, Jaavid Aktar, Raj Dabre, Aswanth Kumar, Ratish Puduppully, and Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2024.acl-short.58/</t>
+          <t>https://aclanthology.org/2024.acl-long.833</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Short Paper</t>
+          <t>Full Paper</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Area Chair Award</t>
         </is>
       </c>
     </row>
@@ -1245,37 +1248,32 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Multilingual</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Utilizing Lexical Similarity to Enable Zero-Shot Machine Translation for Extremely Low-resource Languages</t>
+          <t>NLP/Translation/Evaluation/Indic</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>How Good is Zero-Shot MT Evaluation for Low Resource Indian Languages</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>EACL</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Kaushal Kumar Maurya,  Rahul Kejriwal,  Maunendra Sankar Desarkar,  Anoop Kunchukuttan</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2305.05214</t>
+          <t>ACL</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Anushka Singh, Ananya B. Sai, Raj Dabre, Ratish Puduppully, Anoop Kunchukuttan, Mitesh M Khapra</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>https://aclanthology.org/2024.acl-short.58/</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Short Paper</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>jnoUuGcAAAAJ:VaXvl8Fpj5cC</t>
         </is>
       </c>
     </row>
@@ -1285,82 +1283,82 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>NLP/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>A Comprehensive Analysis of Adapter Efficiency</t>
+          <t>Utilizing Lexical Similarity to Enable Zero-Shot Machine Translation for Extremely Low-resource Languages</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>CoDS-COMAD</t>
+          <t>EACL</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Nandini Mundra,  Sumanth Doddapaneni,  Raj Dabre,  Anoop Kunchukuttan,  Ratish Puduppully,  Mitesh M Khapra</t>
+          <t>Kaushal Kumar Maurya,  Rahul Kejriwal,  Maunendra Sankar Desarkar,  Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2305.07491</t>
+          <t>https://arxiv.org/abs/2305.05214</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Non-archival</t>
+          <t>Short Paper</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:k8Z6L05lTy4C</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>(ES-FoMO Workshop at ICML 2023/non-archival)</t>
+          <t>jnoUuGcAAAAJ:VaXvl8Fpj5cC</t>
         </is>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="4" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>NLP/Transliteration/Evaluation/Multilingual</t>
+          <t>Misc</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Aksharantar: Towards building open transliteration tools for the next billion users</t>
+          <t>A Comprehensive Analysis of Adapter Efficiency</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>EMNLP Findings</t>
+          <t>CoDS-COMAD</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Yash Madhani,  Sushane Parthan,  Priyanka Bedekar,  Ruchi Khapra,  Vivek Seshadri,  Anoop Kunchukuttan,  Pratyush Kumar,  Mitesh M Khapra</t>
+          <t>Nandini Mundra,  Sumanth Doddapaneni,  Raj Dabre,  Anoop Kunchukuttan,  Ratish Puduppully,  Mitesh M Khapra</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2205.03018</t>
+          <t>https://arxiv.org/abs/2305.07491</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Non-archival</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:ML0RJ9NH7IQC</t>
+          <t>jnoUuGcAAAAJ:k8Z6L05lTy4C</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>(ES-FoMO Workshop at ICML 2023/non-archival)</t>
         </is>
       </c>
     </row>
@@ -1370,27 +1368,27 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>NLP/LM/Evaluation/Multilingual/Indic</t>
+          <t>NLP/Transliteration/Evaluation/Multilingual</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Towards Leaving No Indic Language Behind: Building Monolingual Corpora, Benchmark and Models for Indic Languages</t>
+          <t>Aksharantar: Towards building open transliteration tools for the next billion users</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>EMNLP Findings</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Sumanth Doddapaneni,  Rahul Aralikatte,  Gowtham Ramesh,  Shreya Goyal,  Mitesh M Khapra,  Anoop Kunchukuttan,  Pratyush Kumar</t>
+          <t>Yash Madhani,  Sushane Parthan,  Priyanka Bedekar,  Ruchi Khapra,  Vivek Seshadri,  Anoop Kunchukuttan,  Pratyush Kumar,  Mitesh M Khapra</t>
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2023.acl-long.693/</t>
+          <t>https://arxiv.org/abs/2205.03018</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1400,7 +1398,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:gsN89kCJA0AC</t>
+          <t>jnoUuGcAAAAJ:ML0RJ9NH7IQC</t>
         </is>
       </c>
     </row>
@@ -1410,27 +1408,27 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Speech/Indic/ASR</t>
+          <t>NLP/LM/Evaluation/Multilingual/Indic</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Effectiveness of mining audio and text pairs from public data for improving ASR systems for low-resource languages</t>
+          <t>Towards Leaving No Indic Language Behind: Building Monolingual Corpora, Benchmark and Models for Indic Languages</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>ICASSP</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Kaushal Bhogale,  Abhigyan Raman,  Tahir Javed,  Sumanth Doddapaneni,  Anoop Kunchukuttan,  Pratyush Kumar,  Mitesh M Khapra</t>
+          <t>Sumanth Doddapaneni,  Rahul Aralikatte,  Gowtham Ramesh,  Shreya Goyal,  Mitesh M Khapra,  Anoop Kunchukuttan,  Pratyush Kumar</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>https://ieeexplore.ieee.org/abstract/document/10096933/</t>
+          <t>https://aclanthology.org/2023.acl-long.693/</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1440,7 +1438,7 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:tYavs44e6CUC</t>
+          <t>jnoUuGcAAAAJ:gsN89kCJA0AC</t>
         </is>
       </c>
     </row>
@@ -1450,27 +1448,27 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Speech/Indic</t>
+          <t>Speech/Indic/ASR</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>IndicSUPERB: A speech processing universal performance benchmark for indian languages</t>
+          <t>Effectiveness of mining audio and text pairs from public data for improving ASR systems for low-resource languages</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>AAAI</t>
+          <t>ICASSP</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Tahir Javed,  Kaushal Bhogale,  Abhigyan Raman,  Pratyush Kumar,  Anoop Kunchukuttan,  Mitesh M Khapra</t>
+          <t>Kaushal Bhogale,  Abhigyan Raman,  Tahir Javed,  Sumanth Doddapaneni,  Anoop Kunchukuttan,  Pratyush Kumar,  Mitesh M Khapra</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>https://ojs.aaai.org/index.php/AAAI/article/view/26521</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10096933/</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1480,7 +1478,7 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:g3aElNc5_aQC</t>
+          <t>jnoUuGcAAAAJ:tYavs44e6CUC</t>
         </is>
       </c>
     </row>
@@ -1490,27 +1488,27 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>NLP/Indic/Evaluation</t>
+          <t>Speech/Indic</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Naamapadam: A Large-Scale Named Entity Annotated Data for Indic Languages</t>
+          <t>IndicSUPERB: A speech processing universal performance benchmark for indian languages</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>AAAI</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Arnav Mhaske,  Harshit Kedia,  Sumanth Doddapaneni,  Mitesh M Khapra,  Pratyush Kumar,  Rudra Murthy V,  Anoop Kunchukuttan</t>
+          <t>Tahir Javed,  Kaushal Bhogale,  Abhigyan Raman,  Pratyush Kumar,  Anoop Kunchukuttan,  Mitesh M Khapra</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2023.acl-long.582/</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/26521</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1520,7 +1518,7 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:kuK5TVdYjLIC</t>
+          <t>jnoUuGcAAAAJ:g3aElNc5_aQC</t>
         </is>
       </c>
     </row>
@@ -1530,12 +1528,12 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Indic/Evaluation</t>
+          <t>NLP/Indic/Evaluation</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>IndicMT Eval: A Dataset to Meta-Evaluate Machine Translation Metrics for Indian Languages</t>
+          <t>Naamapadam: A Large-Scale Named Entity Annotated Data for Indic Languages</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1545,12 +1543,12 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Ananya Sai B, Tanay Dixit,  Vignesh Nagarajan,  Anoop Kunchukuttan,  Pratyush Kumar,  Mitesh M Khapra,  Raj Dabre</t>
+          <t>Arnav Mhaske,  Harshit Kedia,  Sumanth Doddapaneni,  Mitesh M Khapra,  Pratyush Kumar,  Rudra Murthy V,  Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2023.acl-long.795/</t>
+          <t>https://aclanthology.org/2023.acl-long.582/</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1560,7 +1558,7 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:Ug5p-4gJ2f0C</t>
+          <t>jnoUuGcAAAAJ:kuK5TVdYjLIC</t>
         </is>
       </c>
     </row>
@@ -1570,37 +1568,37 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Indic/Evaluation/Multilingual</t>
+          <t>NLP/Translation/Indic/Evaluation</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>IndicTrans2: Towards High-Quality and Accessible Machine Translation Models for all 22 Scheduled Indian Languages</t>
+          <t>IndicMT Eval: A Dataset to Meta-Evaluate Machine Translation Metrics for Indian Languages</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>TMLR</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Jay Gala,  Pranjal A Chitale,  Raghavan AK,  Sumanth Doddapaneni,  Varun Gumma,  Aswanth Kumar,  Janki Nawale,  Anupama Sujatha,  Ratish Puduppully,  Vivek Raghavan,  Pratyush Kumar,  Mitesh M Khapra,  Raj Dabre,  Anoop Kunchukuttan</t>
+          <t>Ananya Sai B, Tanay Dixit,  Vignesh Nagarajan,  Anoop Kunchukuttan,  Pratyush Kumar,  Mitesh M Khapra,  Raj Dabre</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2305.16307</t>
+          <t>https://aclanthology.org/2023.acl-long.795/</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:M7yex6snE4oC</t>
+          <t>jnoUuGcAAAAJ:Ug5p-4gJ2f0C</t>
         </is>
       </c>
     </row>
@@ -1610,37 +1608,37 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>NLP/Multilingual/Indic/Evaluation</t>
+          <t>NLP/Translation/Indic/Evaluation/Multilingual</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Bhasha-Abhijnaanam: Native-script and romanized Language Identification for 22 Indic languages</t>
+          <t>IndicTrans2: Towards High-Quality and Accessible Machine Translation Models for all 22 Scheduled Indian Languages</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>TMLR</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Yash Madhani,  Mitesh M Khapra,  Anoop Kunchukuttan</t>
+          <t>Jay Gala,  Pranjal A Chitale,  Raghavan AK,  Sumanth Doddapaneni,  Varun Gumma,  Aswanth Kumar,  Janki Nawale,  Anupama Sujatha,  Ratish Puduppully,  Vivek Raghavan,  Pratyush Kumar,  Mitesh M Khapra,  Raj Dabre,  Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2023.acl-short.71/</t>
+          <t>https://arxiv.org/abs/2305.16307</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Short Paper</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:oNZyr7d5Mn4C</t>
+          <t>jnoUuGcAAAAJ:M7yex6snE4oC</t>
         </is>
       </c>
     </row>
@@ -1650,37 +1648,37 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>NLP/LM/Translation/Multilingual</t>
+          <t>NLP/Multilingual/Indic/Evaluation</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Decomposed Prompting for Machine Translation Between Related Languages using Large Language Models</t>
+          <t>Bhasha-Abhijnaanam: Native-script and romanized Language Identification for 22 Indic languages</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>EMNLP</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Ratish Puduppully,  Anoop Kunchukuttan,  Raj Dabre,  Ai Ti Aw,  Nancy F Chen</t>
+          <t>Yash Madhani,  Mitesh M Khapra,  Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2305.13085</t>
+          <t>https://aclanthology.org/2023.acl-short.71/</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Short Paper</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:hCrLmN-GePgC</t>
+          <t>jnoUuGcAAAAJ:oNZyr7d5Mn4C</t>
         </is>
       </c>
     </row>
@@ -1690,27 +1688,27 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>NLP/LM/Translation</t>
+          <t>NLP/LM/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>In-context Example Selection for Machine Translation Using Multiple Features</t>
+          <t>Decomposed Prompting for Machine Translation Between Related Languages using Large Language Models</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>EMNLP Findings</t>
+          <t>EMNLP</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Aswanth Kumar,  Ratish Puduppully,  Raj Dabre,  Anoop Kunchukuttan</t>
+          <t>Ratish Puduppully,  Anoop Kunchukuttan,  Raj Dabre,  Ai Ti Aw,  Nancy F Chen</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2305.14105</t>
+          <t>https://arxiv.org/abs/2305.13085</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1720,7 +1718,7 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:kz9GbA2Ns4gC</t>
+          <t>jnoUuGcAAAAJ:hCrLmN-GePgC</t>
         </is>
       </c>
     </row>
@@ -1730,80 +1728,79 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>NLP/Indic</t>
+          <t>NLP/LM/Translation</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Evaluating Inter-Bilingual Semantic Parsing for Indian Languages</t>
+          <t>In-context Example Selection for Machine Translation Using Multiple Features</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>NLP4ConvAI</t>
+          <t>EMNLP Findings</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Divyanshu Aggarwal,  Vivek Gupta,  Anoop Kunchukuttan</t>
+          <t>Aswanth Kumar,  Ratish Puduppully,  Raj Dabre,  Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2023.nlp4convai-1.9/</t>
+          <t>https://arxiv.org/abs/2305.14105</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:LI9QrySNdTsC</t>
+          <t>jnoUuGcAAAAJ:kz9GbA2Ns4gC</t>
         </is>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
       <c r="A33" s="4" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Indic/Multilingual</t>
+          <t>NLP/Indic</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Samanantar: The largest publicly available parallel corpora collection for 11 Indic languages</t>
+          <t>Evaluating Inter-Bilingual Semantic Parsing for Indian Languages</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>TACL</t>
+          <t>NLP4ConvAI</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Gowtham Ramesh,  Sumanth Doddapaneni,  Aravinth Bheemaraj,  Mayank Jobanputra,  Raghavan AK,  Ajitesh Sharma,  Sujit Sahoo,  Harshita Diddee,  Divyanshu Kakwani,  Navneet Kumar,  Aswin Pradeep,  Kumar Deepak,  Vivek Raghavan,  Anoop Kunchukuttan,  Pratyush Kumar,  Mitesh Shantadevi Khapra</t>
+          <t>Divyanshu Aggarwal,  Vivek Gupta,  Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>https://direct.mit.edu/tacl/article-abstract/doi/10.1162/tacl_a_00452/109468</t>
+          <t>https://aclanthology.org/2023.nlp4convai-1.9/</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:j8SEvjWlNXcC</t>
-        </is>
-      </c>
-      <c r="J33" s="7" t="n"/>
+          <t>jnoUuGcAAAAJ:LI9QrySNdTsC</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="60" customHeight="1">
       <c r="A34" s="4" t="n">
@@ -1811,37 +1808,37 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>NLP/LM/Indic</t>
+          <t>NLP/Translation/Indic/Multilingual</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>IndicBART: A Pre-trained Model for Indic Natural Language Generation</t>
+          <t>Samanantar: The largest publicly available parallel corpora collection for 11 Indic languages</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>ACL Findings</t>
+          <t>TACL</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Raj Dabre,  Himani Shrotriya,  Anoop Kunchukuttan,  Ratish Puduppully,  Mitesh M Khapra,  Pratyush Kumar</t>
+          <t>Gowtham Ramesh,  Sumanth Doddapaneni,  Aravinth Bheemaraj,  Mayank Jobanputra,  Raghavan AK,  Ajitesh Sharma,  Sujit Sahoo,  Harshita Diddee,  Divyanshu Kakwani,  Navneet Kumar,  Aswin Pradeep,  Kumar Deepak,  Vivek Raghavan,  Anoop Kunchukuttan,  Pratyush Kumar,  Mitesh Shantadevi Khapra</t>
         </is>
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2022.findings-acl.145/</t>
+          <t>https://direct.mit.edu/tacl/article-abstract/doi/10.1162/tacl_a_00452/109468</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:XoXfffV-tXoC</t>
+          <t>jnoUuGcAAAAJ:j8SEvjWlNXcC</t>
         </is>
       </c>
       <c r="J34" s="7" t="n"/>
@@ -1852,27 +1849,27 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Speech/ASR/Indic</t>
+          <t>NLP/LM/Indic</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Towards Building ASR Systems for the Next Billion Users</t>
+          <t>IndicBART: A Pre-trained Model for Indic Natural Language Generation</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>AAAI</t>
+          <t>ACL Findings</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Tahir Javed,  Sumanth Doddapaneni,  Abhigyan Raman,  Kaushal Santosh Bhogale,  Gowtham Ramesh,  Anoop Kunchukuttan,  Pratyush Kumar,  Mitesh M Khapra</t>
+          <t>Raj Dabre,  Himani Shrotriya,  Anoop Kunchukuttan,  Ratish Puduppully,  Mitesh M Khapra,  Pratyush Kumar</t>
         </is>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>https://ojs.aaai.org/index.php/AAAI/article/view/21327</t>
+          <t>https://aclanthology.org/2022.findings-acl.145/</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1882,7 +1879,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:epqYDVWIO7EC</t>
+          <t>jnoUuGcAAAAJ:XoXfffV-tXoC</t>
         </is>
       </c>
       <c r="J35" s="7" t="n"/>
@@ -1893,27 +1890,27 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>NLP/LM/Evaluation/Multilingual</t>
+          <t>Speech/ASR/Indic</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>IndicNLG benchmark: Multilingual datasets for diverse NLG tasks in indic languages</t>
+          <t>Towards Building ASR Systems for the Next Billion Users</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>EMNLP</t>
+          <t>AAAI</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Aman Kumar,  Himani Shrotriya,  Prachi Sahu,  Amogh Mishra,  Raj Dabre,  Ratish Puduppully,  Anoop Kunchukuttan,  Mitesh M Khapra,  Pratyush Kumar</t>
+          <t>Tahir Javed,  Sumanth Doddapaneni,  Abhigyan Raman,  Kaushal Santosh Bhogale,  Gowtham Ramesh,  Anoop Kunchukuttan,  Pratyush Kumar,  Mitesh M Khapra</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2022.emnlp-main.360/</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/21327</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1923,7 +1920,7 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:MLfJN-KU85MC</t>
+          <t>jnoUuGcAAAAJ:epqYDVWIO7EC</t>
         </is>
       </c>
       <c r="J36" s="7" t="n"/>
@@ -1934,12 +1931,12 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>NLP/Indic</t>
+          <t>NLP/LM/Evaluation/Multilingual</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>IndicXNLI: Evaluating multilingual inference for Indian languages</t>
+          <t>IndicNLG benchmark: Multilingual datasets for diverse NLG tasks in indic languages</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1949,12 +1946,12 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Divyanshu Aggarwal,  Vivek Gupta,  Anoop Kunchukuttan</t>
+          <t>Aman Kumar,  Himani Shrotriya,  Prachi Sahu,  Amogh Mishra,  Raj Dabre,  Ratish Puduppully,  Anoop Kunchukuttan,  Mitesh M Khapra,  Pratyush Kumar</t>
         </is>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2022.emnlp-main.755/</t>
+          <t>https://aclanthology.org/2022.emnlp-main.360/</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1964,7 +1961,7 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:Z5m8FVwuT1cC</t>
+          <t>jnoUuGcAAAAJ:MLfJN-KU85MC</t>
         </is>
       </c>
       <c r="J37" s="7" t="n"/>
@@ -1980,22 +1977,22 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Bilingual tabular inference: A case study on indic languages</t>
+          <t>IndicXNLI: Evaluating multilingual inference for Indian languages</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>NAACL</t>
+          <t>EMNLP</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Chaitanya Agarwal,  Vivek Gupta,  Anoop Kunchukuttan,  Manish Shrivastava</t>
+          <t>Divyanshu Aggarwal,  Vivek Gupta,  Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2022.naacl-main.295/</t>
+          <t>https://aclanthology.org/2022.emnlp-main.755/</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -2005,14 +2002,14 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:BwyfMAYsbu0C</t>
+          <t>jnoUuGcAAAAJ:Z5m8FVwuT1cC</t>
         </is>
       </c>
       <c r="J38" s="7" t="n"/>
     </row>
     <row r="39" ht="60" customHeight="1">
       <c r="A39" s="4" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
@@ -2021,34 +2018,35 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>The AI4Bharat Initiative</t>
+          <t>Bilingual tabular inference: A case study on indic languages</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>ICON 2021</t>
+          <t>NAACL</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan, Mitesh Khapra, Pratyush Kumar</t>
-        </is>
-      </c>
-      <c r="F39" s="1" t="inlineStr">
-        <is>
-          <t>https://anoopkunchukuttan.gitlab.io/publications/presentations/AI4Bharat_Initiative_ICON2021.pdf</t>
+          <t>Chaitanya Agarwal,  Vivek Gupta,  Anoop Kunchukuttan,  Manish Shrivastava</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>https://aclanthology.org/2022.naacl-main.295/</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Tutorial</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:umqufdRvDiIC</t>
-        </is>
-      </c>
+          <t>jnoUuGcAAAAJ:BwyfMAYsbu0C</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="n"/>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="4" t="n">
@@ -2056,40 +2054,39 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>NLP/Transliteration/Indic/Multilingual</t>
+          <t>NLP/Indic</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>A large-scale evaluation of neural machine transliteration for indic languages</t>
+          <t>The AI4Bharat Initiative</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>EACL</t>
+          <t>ICON 2021</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Siddharth Jain,  Rahul Kejriwal</t>
-        </is>
-      </c>
-      <c r="F40" s="10" t="inlineStr">
-        <is>
-          <t>https://aclanthology.org/2021.eacl-main.303/</t>
+          <t>Anoop Kunchukuttan, Mitesh Khapra, Pratyush Kumar</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
+        <is>
+          <t>https://anoopkunchukuttan.gitlab.io/publications/presentations/AI4Bharat_Initiative_ICON2021.pdf</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Short Paper</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:uJ-U7cs_P_0C</t>
-        </is>
-      </c>
-      <c r="J40" s="7" t="n"/>
+          <t>jnoUuGcAAAAJ:umqufdRvDiIC</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="4" t="n">
@@ -2097,37 +2094,37 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Transliteration/Indic/Multilingual</t>
+          <t>NLP/Transliteration/Indic/Multilingual</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Machine Translation and Transliteration involving Related, Low-resource Languages</t>
+          <t>A large-scale evaluation of neural machine transliteration for indic languages</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>CRC Press</t>
+          <t>EACL</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan, Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Siddharth Jain,  Rahul Kejriwal</t>
         </is>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.in/Translation-Transliteration-involving-Low-resource-Languages/dp/0367561999</t>
+          <t>https://aclanthology.org/2021.eacl-main.303/</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Book</t>
+          <t>Short Paper</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:XvxMoLDsR5gC</t>
+          <t>jnoUuGcAAAAJ:uJ-U7cs_P_0C</t>
         </is>
       </c>
       <c r="J41" s="7" t="n"/>
@@ -2138,37 +2135,37 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Multilingual</t>
+          <t>NLP/Translation/Transliteration/Indic/Multilingual</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>An Empirical Investigation of Multi-bridge Multilingual NMT models</t>
+          <t>Machine Translation and Transliteration involving Related, Low-resource Languages</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>arXiv preprint arXiv:2110.07304</t>
+          <t>CRC Press</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan</t>
+          <t>Anoop Kunchukuttan, Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2110.07304</t>
+          <t>https://www.amazon.in/Translation-Transliteration-involving-Low-resource-Languages/dp/0367561999</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Book</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:zLWjf1WUPmwC</t>
+          <t>jnoUuGcAAAAJ:XvxMoLDsR5gC</t>
         </is>
       </c>
       <c r="J42" s="7" t="n"/>
@@ -2179,37 +2176,37 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Indic</t>
+          <t>NLP/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Itihasa: A large-scale corpus for Sanskrit to English translation</t>
+          <t>An Empirical Investigation of Multi-bridge Multilingual NMT models</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>WAT</t>
+          <t>arXiv preprint arXiv:2110.07304</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Rahul Aralikatte,  Miryam de Lhoneux,  Anoop Kunchukuttan,  Anders Søgaard</t>
+          <t>Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2021.wat-1.22/</t>
+          <t>https://arxiv.org/abs/2110.07304</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:VLnqNzywnoUC</t>
+          <t>jnoUuGcAAAAJ:zLWjf1WUPmwC</t>
         </is>
       </c>
       <c r="J43" s="7" t="n"/>
@@ -2220,12 +2217,12 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Translation/Indic</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Proceedings of the 8th Workshop on Asian Translation (WAT2021)</t>
+          <t>Itihasa: A large-scale corpus for Sanskrit to English translation</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -2235,63 +2232,63 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Toshiaki Nakazawa,  Hideki Nakayama,  Isao Goto,  Hideya Mino,  Chenchen Ding,  Raj Dabre,  Anoop Kunchukuttan,  Shohei Higashiyama,  Hiroshi Manabe,  Win Pa Pa,  Shantipriya Parida,  Ondřej Bojar,  Chenhui Chu,  Akiko Eriguchi,  Kaori Abe,  Yusuke Oda,  Katsuhito Sudoh,  Sadao Kurohashi,  Pushpak Bhattacharyya</t>
+          <t>Rahul Aralikatte,  Miryam de Lhoneux,  Anoop Kunchukuttan,  Anders Søgaard</t>
         </is>
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2021.wat-1.0.pdf</t>
+          <t>https://aclanthology.org/2021.wat-1.22/</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Proceedings</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:vDijr-p_gm4C</t>
+          <t>jnoUuGcAAAAJ:VLnqNzywnoUC</t>
         </is>
       </c>
       <c r="J44" s="7" t="n"/>
     </row>
     <row r="45" ht="75" customHeight="1">
       <c r="A45" s="4" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>NLP/LM/Indic/Evaluation/Embeddings</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>IndicNLPSuite: Monolingual Corpora, Evaluation Benchmarks and Pre-trained Multilingual Language Models for Indian Languages.</t>
+          <t>Proceedings of the 8th Workshop on Asian Translation (WAT2021)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>EMNLP Findings</t>
+          <t>WAT</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Divyanshu Kakwani,  Anoop Kunchukuttan,  Satish Golla,  Gokul N.C.,  Avik Bhattacharyya,  Mitesh M. Khapra,  Pratyush Kumar</t>
+          <t>Toshiaki Nakazawa,  Hideki Nakayama,  Isao Goto,  Hideya Mino,  Chenchen Ding,  Raj Dabre,  Anoop Kunchukuttan,  Shohei Higashiyama,  Hiroshi Manabe,  Win Pa Pa,  Shantipriya Parida,  Ondřej Bojar,  Chenhui Chu,  Akiko Eriguchi,  Kaori Abe,  Yusuke Oda,  Katsuhito Sudoh,  Sadao Kurohashi,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2020.findings-emnlp.445/</t>
+          <t>https://aclanthology.org/2021.wat-1.0.pdf</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Proceedings</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:dQ2og3OwTAUC</t>
+          <t>jnoUuGcAAAAJ:vDijr-p_gm4C</t>
         </is>
       </c>
       <c r="J45" s="7" t="n"/>
@@ -2302,37 +2299,37 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Multilingual</t>
+          <t>NLP/LM/Indic/Evaluation/Embeddings</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>A Survey of Multilingual Neural Machine Translation</t>
+          <t>IndicNLPSuite: Monolingual Corpora, Evaluation Benchmarks and Pre-trained Multilingual Language Models for Indian Languages.</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>ACM Computing Surveys</t>
+          <t>EMNLP Findings</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Raj Dabre,  Chenhui Chu,  Anoop Kunchukuttan</t>
+          <t>Divyanshu Kakwani,  Anoop Kunchukuttan,  Satish Golla,  Gokul N.C.,  Avik Bhattacharyya,  Mitesh M. Khapra,  Pratyush Kumar</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t>https://dl.acm.org/doi/abs/10.1145/3406095</t>
+          <t>https://aclanthology.org/2020.findings-emnlp.445/</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:WqliGbK-hY8C</t>
+          <t>jnoUuGcAAAAJ:dQ2og3OwTAUC</t>
         </is>
       </c>
       <c r="J46" s="7" t="n"/>
@@ -2343,37 +2340,37 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Overview of the 7th Workshop on Asian Translation</t>
+          <t>A Survey of Multilingual Neural Machine Translation</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>WAT</t>
+          <t>ACM Computing Surveys</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Toshiaki Nakazawa,  Hideki Nakayama,  Chenchen Ding,  Raj Dabre,  Shohei Higashiyama,  Hideya Mino,  Isao Goto,  Win Pa Pa,  Anoop Kunchukuttan,  Shantipriya Parida,  Ondřej Bojar,  Sadao Kurohashi</t>
+          <t>Raj Dabre,  Chenhui Chu,  Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2021.wat-1.1/</t>
+          <t>https://dl.acm.org/doi/abs/10.1145/3406095</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Survey</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:-_dYPAW6P2MC</t>
+          <t>jnoUuGcAAAAJ:WqliGbK-hY8C</t>
         </is>
       </c>
       <c r="J47" s="7" t="n"/>
@@ -2384,37 +2381,37 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>NLP/Indic</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Indic NLP Library: A unified approach to NLP for Indian languages</t>
+          <t>Overview of the 7th Workshop on Asian Translation</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>WAT</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan</t>
-        </is>
-      </c>
-      <c r="F48" s="1" t="inlineStr">
-        <is>
-          <t>https://github.com/anoopkunchukuttan/indic_nlp_library/blob/master/docs/indicnlp.pdf</t>
+          <t>Toshiaki Nakazawa,  Hideki Nakayama,  Chenchen Ding,  Raj Dabre,  Shohei Higashiyama,  Hideya Mino,  Isao Goto,  Win Pa Pa,  Anoop Kunchukuttan,  Shantipriya Parida,  Ondřej Bojar,  Sadao Kurohashi</t>
+        </is>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>https://aclanthology.org/2021.wat-1.1/</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:ZuybSZzF8UAC</t>
+          <t>jnoUuGcAAAAJ:-_dYPAW6P2MC</t>
         </is>
       </c>
       <c r="J48" s="7" t="n"/>
@@ -2425,37 +2422,37 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>NLP/Embeddings/Indic</t>
+          <t>NLP/Indic</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>AI4Bharat-IndicNLP corpus: Monolingual corpora and word embeddings for Indic languages</t>
+          <t>Indic NLP Library: A unified approach to NLP for Indian languages</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>REPL4NLP/non-archival</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Divyanshu Kakwani,  Satish Golla,  Avik Bhattacharyya,  Mitesh M Khapra,  Pratyush Kumar</t>
-        </is>
-      </c>
-      <c r="F49" s="10" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2005.00085</t>
+          <t>Anoop Kunchukuttan</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>https://github.com/anoopkunchukuttan/indic_nlp_library/blob/master/docs/indicnlp.pdf</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>Non-archival</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:PR6Y55bgFSsC</t>
+          <t>jnoUuGcAAAAJ:ZuybSZzF8UAC</t>
         </is>
       </c>
       <c r="J49" s="7" t="n"/>
@@ -2466,37 +2463,37 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Indic/Multilingual</t>
+          <t>NLP/Embeddings/Indic</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Utilizing language relatedness to improve machine translation: A case study on languages of the indian subcontinent</t>
+          <t>AI4Bharat-IndicNLP corpus: Monolingual corpora and word embeddings for Indic languages</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>arXiv preprint arXiv:2003.08925</t>
+          <t>REPL4NLP/non-archival</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Divyanshu Kakwani,  Satish Golla,  Avik Bhattacharyya,  Mitesh M Khapra,  Pratyush Kumar</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2003.08925</t>
+          <t>https://arxiv.org/abs/2005.00085</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Non-archival</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:VL0QpB8kHFEC</t>
+          <t>jnoUuGcAAAAJ:PR6Y55bgFSsC</t>
         </is>
       </c>
       <c r="J50" s="7" t="n"/>
@@ -2507,37 +2504,37 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>NLP/Embeddings</t>
+          <t>NLP/Translation/Indic/Multilingual</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Learning Geometric Word Meta-Embeddings</t>
+          <t>Utilizing language relatedness to improve machine translation: A case study on languages of the indian subcontinent</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>REPL4NLP</t>
+          <t>arXiv preprint arXiv:2003.08925</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Pratik Jawanpuria,  NTV Dev,  Anoop Kunchukuttan,  Bamdev Mishra</t>
+          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2020.repl4nlp-1.6/</t>
+          <t>https://arxiv.org/abs/2003.08925</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:1yQoGdGgb4wC</t>
+          <t>jnoUuGcAAAAJ:VL0QpB8kHFEC</t>
         </is>
       </c>
       <c r="J51" s="7" t="n"/>
@@ -2548,37 +2545,37 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Indic</t>
+          <t>NLP/Embeddings</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Contact Relatedness can help improve multilingual NMT: Microsoft STCI-MT @ WMT20</t>
+          <t>Learning Geometric Word Meta-Embeddings</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>REPL4NLP</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Vikrant Goyal,  Anoop Kunchukuttan,  Rahul Kejriwal,  Siddharth Jain,  Amit Bhagwat</t>
+          <t>Pratik Jawanpuria,  NTV Dev,  Anoop Kunchukuttan,  Bamdev Mishra</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2020.wmt-1.19/</t>
+          <t>https://aclanthology.org/2020.repl4nlp-1.6/</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>Shared Task</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:2KloaMYe4IUC</t>
+          <t>jnoUuGcAAAAJ:1yQoGdGgb4wC</t>
         </is>
       </c>
       <c r="J52" s="7" t="n"/>
@@ -2594,32 +2591,32 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>The IndoWordnet Parallel Corpus</t>
+          <t>Contact Relatedness can help improve multilingual NMT: Microsoft STCI-MT @ WMT20</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/anoopkunchukuttan/indowordnet_parallel/blob/master/iwn_parallel_2020.pdf</t>
+          <t>Vikrant Goyal,  Anoop Kunchukuttan,  Rahul Kejriwal,  Siddharth Jain,  Amit Bhagwat</t>
+        </is>
+      </c>
+      <c r="F53" s="10" t="inlineStr">
+        <is>
+          <t>https://aclanthology.org/2020.wmt-1.19/</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Shared Task</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:N5tVd3kTz84C</t>
+          <t>jnoUuGcAAAAJ:2KloaMYe4IUC</t>
         </is>
       </c>
       <c r="J53" s="7" t="n"/>
@@ -2630,78 +2627,78 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Multilingual</t>
+          <t>NLP/Translation/Indic</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Multilingual neural machine translation</t>
+          <t>The IndoWordnet Parallel Corpus</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>COLING</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Raj Dabre,  Chenhui Chu,  Anoop Kunchukuttan</t>
-        </is>
-      </c>
-      <c r="F54" s="10" t="inlineStr">
-        <is>
-          <t>https://aclanthology.org/2020.coling-tutorials.3/</t>
+          <t>Anoop Kunchukuttan</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/anoopkunchukuttan/indowordnet_parallel/blob/master/iwn_parallel_2020.pdf</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>Tutorial</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:35r97b3x0nAC</t>
+          <t>jnoUuGcAAAAJ:N5tVd3kTz84C</t>
         </is>
       </c>
       <c r="J54" s="7" t="n"/>
     </row>
     <row r="55" ht="60" customHeight="1">
       <c r="A55" s="4" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>NLP/Embeddings/Multilingual</t>
+          <t>NLP/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Learning multilingual word embeddings in latent metric space: a geometric approach</t>
+          <t>Multilingual neural machine translation</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>TACL</t>
+          <t>COLING</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>Pratik Jawanpuria,  Arjun Balgovind,  Anoop Kunchukuttan,  Bamdev Mishra</t>
+          <t>Raj Dabre,  Chenhui Chu,  Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t>https://direct.mit.edu/tacl/article-abstract/doi/10.1162/tacl_a_00257/43509</t>
+          <t>https://aclanthology.org/2020.coling-tutorials.3/</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:AXPGKjj_ei8C</t>
+          <t>jnoUuGcAAAAJ:35r97b3x0nAC</t>
         </is>
       </c>
       <c r="J55" s="7" t="n"/>
@@ -2712,37 +2709,37 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Multilingual</t>
+          <t>NLP/Embeddings/Multilingual</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Addressing word-order Divergence in Multilingual Neural Machine Translation for extremely Low Resource Languages</t>
+          <t>Learning multilingual word embeddings in latent metric space: a geometric approach</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>NAACL</t>
+          <t>TACL</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>Rudra Murthy V,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Pratik Jawanpuria,  Arjun Balgovind,  Anoop Kunchukuttan,  Bamdev Mishra</t>
         </is>
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/N19-1387/</t>
+          <t>https://direct.mit.edu/tacl/article-abstract/doi/10.1162/tacl_a_00257/43509</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>Short Paper</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:tkaPQYYpVKoC</t>
+          <t>jnoUuGcAAAAJ:AXPGKjj_ei8C</t>
         </is>
       </c>
       <c r="J56" s="7" t="n"/>
@@ -2753,78 +2750,78 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Proceedings of the 6th Workshop on Asian Translation</t>
+          <t>Addressing word-order Divergence in Multilingual Neural Machine Translation for extremely Low Resource Languages</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>WAT</t>
+          <t>NAACL</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>Toshiaki Nakazawa,  Chenchen Ding,  Raj Dabre,  Anoop Kunchukuttan,  Nobushige Doi,  Yusuke Oda,  Ondřej Bojar,  Shantipriya Parida,  Isao Goto,  Hidaya Mino</t>
+          <t>Rudra Murthy V,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/D19-5200.pdf</t>
+          <t>https://aclanthology.org/N19-1387/</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>Proceedings</t>
+          <t>Short Paper</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:5awf1xo2G04C</t>
+          <t>jnoUuGcAAAAJ:tkaPQYYpVKoC</t>
         </is>
       </c>
       <c r="J57" s="7" t="n"/>
     </row>
     <row r="58" ht="60" customHeight="1">
       <c r="A58" s="4" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Indic</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>The IIT Bombay English-Hindi Parallel Corpus</t>
+          <t>Proceedings of the 6th Workshop on Asian Translation</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>LREC</t>
+          <t>WAT</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Pratik Mehta,  Pushpak Bhattacharyya</t>
+          <t>Toshiaki Nakazawa,  Chenchen Ding,  Raj Dabre,  Anoop Kunchukuttan,  Nobushige Doi,  Yusuke Oda,  Ondřej Bojar,  Shantipriya Parida,  Isao Goto,  Hidaya Mino</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/L18-1548/</t>
+          <t>https://aclanthology.org/D19-5200.pdf</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Proceedings</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:bnK-pcrLprsC</t>
+          <t>jnoUuGcAAAAJ:5awf1xo2G04C</t>
         </is>
       </c>
       <c r="J58" s="7" t="n"/>
@@ -2835,37 +2832,37 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>NLP/Translation/Indic</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>McTorch, a manifold optimization library for deep learning</t>
+          <t>The IIT Bombay English-Hindi Parallel Corpus</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Workshop on Machine Learning Open Source Software @NIPS</t>
+          <t>LREC</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>Mayank Meghwanshi,  Pratik Jawanpuria,  Anoop Kunchukuttan,  Hiroyuki Kasai,  Bamdev Mishra</t>
+          <t>Anoop Kunchukuttan,  Pratik Mehta,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/1810.01811</t>
+          <t>https://aclanthology.org/L18-1548/</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:Y5dfb0dijaUC</t>
+          <t>jnoUuGcAAAAJ:bnK-pcrLprsC</t>
         </is>
       </c>
       <c r="J59" s="7" t="n"/>
@@ -2876,37 +2873,37 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>NLP/Transliteration/Multilingual/Indic</t>
+          <t>Misc</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Leveraging Orthographic Similarity for Multilingual Neural Transliteration</t>
+          <t>McTorch, a manifold optimization library for deep learning</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>TACL</t>
+          <t>Workshop on Machine Learning Open Source Software @NIPS</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Mitesh Khapra,  Gurneet Singh,  Pushpak Bhattacharyya</t>
+          <t>Mayank Meghwanshi,  Pratik Jawanpuria,  Anoop Kunchukuttan,  Hiroyuki Kasai,  Bamdev Mishra</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t>https://direct.mit.edu/tacl/article-abstract/doi/10.1162/tacl_a_00022/43438</t>
+          <t>https://arxiv.org/abs/1810.01811</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:olpn-zPbct0C</t>
+          <t>jnoUuGcAAAAJ:Y5dfb0dijaUC</t>
         </is>
       </c>
       <c r="J60" s="7" t="n"/>
@@ -2917,37 +2914,37 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>NLP/Multilingual</t>
+          <t>NLP/Transliteration/Multilingual/Indic</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Judicious Selection of Training Data in Assisting Language for Multilingual Neural NER</t>
+          <t>Leveraging Orthographic Similarity for Multilingual Neural Transliteration</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>TACL</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>V Rudramurthy,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Mitesh Khapra,  Gurneet Singh,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/P18-2064/</t>
+          <t>https://direct.mit.edu/tacl/article-abstract/doi/10.1162/tacl_a_00022/43438</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>Short Paper</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:WA5NYHcadZ8C</t>
+          <t>jnoUuGcAAAAJ:olpn-zPbct0C</t>
         </is>
       </c>
       <c r="J61" s="7" t="n"/>
@@ -2958,37 +2955,37 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Multilingual</t>
+          <t>NLP/Multilingual</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>NICT's Participation in WAT 2018: Approaches Using Multilingualism and Recurrently Stacked Layers.</t>
+          <t>Judicious Selection of Training Data in Assisting Language for Multilingual Neural NER</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>WAT</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>Raj Dabre,  Anoop Kunchukuttan,  Atsushi Fujita,  Eiichiro Sumita</t>
+          <t>V Rudramurthy,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/Y18-3003.pdf</t>
+          <t>https://aclanthology.org/P18-2064/</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>Shared Task</t>
+          <t>Short Paper</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:_B80troHkn4C</t>
+          <t>jnoUuGcAAAAJ:WA5NYHcadZ8C</t>
         </is>
       </c>
       <c r="J62" s="7" t="n"/>
@@ -3004,7 +3001,7 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Multilingual Indian Language Translation System at WAT 2018: Many-to-one Phrase-based SMT</t>
+          <t>NICT's Participation in WAT 2018: Approaches Using Multilingualism and Recurrently Stacked Layers.</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -3014,12 +3011,12 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>Tamali Banerjee,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Raj Dabre,  Anoop Kunchukuttan,  Atsushi Fujita,  Eiichiro Sumita</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/Y18-3013.pdf</t>
+          <t>https://aclanthology.org/Y18-3003.pdf</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -3029,7 +3026,7 @@
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:PELIpwtuRlgC</t>
+          <t>jnoUuGcAAAAJ:_B80troHkn4C</t>
         </is>
       </c>
       <c r="J63" s="7" t="n"/>
@@ -3040,37 +3037,37 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Transliteration/Indic/Multilingual</t>
+          <t>NLP/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Machine Translation and Transliteration involving Related, Low-resource Languages</t>
+          <t>Multilingual Indian Language Translation System at WAT 2018: Many-to-one Phrase-based SMT</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>IIT Bombay</t>
+          <t>WAT</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan</t>
+          <t>Tamali Banerjee,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>https://aclanthology.org/Y18-3013.pdf</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>Thesis</t>
+          <t>Shared Task</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:JoZmwDi-zQgC</t>
+          <t>jnoUuGcAAAAJ:PELIpwtuRlgC</t>
         </is>
       </c>
       <c r="J64" s="7" t="n"/>
@@ -3081,22 +3078,22 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Translation/Transliteration/Indic/Multilingual</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Overview of the 5th Workshop on Asian Translation</t>
+          <t>Machine Translation and Transliteration involving Related, Low-resource Languages</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>WAT</t>
+          <t>IIT Bombay</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>Toshiaki Nakazawa,  Shohei Higashiyama,  Chenchen Ding,  Raj Dabre,  Anoop Kunchukuttan,  Win Pa Pa,  Isao Goto,  Hideya Mino,  Katsuhito Sudoh,  Sadao Kurohashi</t>
+          <t>Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F65" s="10" t="inlineStr">
@@ -3106,55 +3103,56 @@
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>Proceedings</t>
+          <t>Thesis</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:dTyEYWd-f8wC</t>
+          <t>jnoUuGcAAAAJ:JoZmwDi-zQgC</t>
         </is>
       </c>
       <c r="J65" s="7" t="n"/>
     </row>
     <row r="66" ht="45" customHeight="1">
       <c r="A66" s="4" t="n">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Multilingual</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Learning variable length units for SMT between related languages via Byte Pair Encoding</t>
+          <t>Overview of the 5th Workshop on Asian Translation</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>First Workshop on Subword and Character LEvel Models in NLP (SCLeM)</t>
+          <t>WAT</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Toshiaki Nakazawa,  Shohei Higashiyama,  Chenchen Ding,  Raj Dabre,  Anoop Kunchukuttan,  Win Pa Pa,  Isao Goto,  Hideya Mino,  Katsuhito Sudoh,  Sadao Kurohashi</t>
         </is>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/1610.06510</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Proceedings</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:BrmTIyaxlBUC</t>
-        </is>
-      </c>
+          <t>jnoUuGcAAAAJ:dTyEYWd-f8wC</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="n"/>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="4" t="n">
@@ -3162,37 +3160,37 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Comparing Recurrent and Convolutional Architectures for English-Hindi Neural Machine Translation</t>
+          <t>Learning variable length units for SMT between related languages via Byte Pair Encoding</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>WAT</t>
+          <t>First Workshop on Subword and Character LEvel Models in NLP (SCLeM)</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>Sandhya Singh,  Ritesh Panjwani,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W17-5717/</t>
+          <t>https://arxiv.org/abs/1610.06510</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>Shared Task</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:XiVPGOgt02cC</t>
+          <t>jnoUuGcAAAAJ:BrmTIyaxlBUC</t>
         </is>
       </c>
     </row>
@@ -3202,67 +3200,67 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Multilingual</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Utilizing Lexical Similarity between Related, Low-resource Languages for Pivot-based SMT</t>
+          <t>Comparing Recurrent and Convolutional Architectures for English-Hindi Neural Machine Translation</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>IJCNLP</t>
+          <t>WAT</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Maulik Shah,  Pradyot Prakash,  Pushpak Bhattacharyya</t>
+          <t>Sandhya Singh,  Ritesh Panjwani,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/1702.07203</t>
+          <t>https://aclanthology.org/W17-5717/</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>Short Paper</t>
+          <t>Shared Task</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:q3oQSFYPqjQC</t>
+          <t>jnoUuGcAAAAJ:XiVPGOgt02cC</t>
         </is>
       </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="4" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Indic/Multilingual</t>
+          <t>NLP/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Orthographic Syllable as basic unit for SMT between Related Languages</t>
+          <t>Utilizing Lexical Similarity between Related, Low-resource Languages for Pivot-based SMT</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>EMNLP</t>
+          <t>IJCNLP</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Maulik Shah,  Pradyot Prakash,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/1610.00634</t>
+          <t>https://arxiv.org/abs/1702.07203</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -3272,7 +3270,7 @@
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:D_sINldO8mEC</t>
+          <t>jnoUuGcAAAAJ:q3oQSFYPqjQC</t>
         </is>
       </c>
     </row>
@@ -3282,37 +3280,37 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Multilingual</t>
+          <t>NLP/Translation/Indic/Multilingual</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Statistical machine translation between related languages</t>
+          <t>Orthographic Syllable as basic unit for SMT between Related Languages</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>NAACL Tutorial</t>
+          <t>EMNLP</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>Pushpak Bhattacharyya,  Mitesh M Khapra,  Anoop Kunchukuttan</t>
+          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/N16-4006.pdf</t>
+          <t>https://arxiv.org/abs/1610.00634</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>Tutorial</t>
+          <t>Short Paper</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:5ugPr518TE4C</t>
+          <t>jnoUuGcAAAAJ:D_sINldO8mEC</t>
         </is>
       </c>
     </row>
@@ -3322,37 +3320,37 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Faster decoding for subword level Phrase-based SMT between related languages.</t>
+          <t>Statistical machine translation between related languages</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Third Workshop on NLP for Similar Languages, Varieties and Dialects</t>
+          <t>NAACL Tutorial</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Pushpak Bhattacharyya,  Mitesh M Khapra,  Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/1611.00354</t>
+          <t>https://aclanthology.org/N16-4006.pdf</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:eflP2zaiRacC</t>
+          <t>jnoUuGcAAAAJ:5ugPr518TE4C</t>
         </is>
       </c>
     </row>
@@ -3362,37 +3360,37 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>NLP/Transliteration</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Substring-based Unsupervised Transliteration with Phonetic and Contextual Knowledge</t>
+          <t>Faster decoding for subword level Phrase-based SMT between related languages.</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>CoNLL</t>
+          <t>Third Workshop on NLP for Similar Languages, Varieties and Dialects</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Mitesh Khapra Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/K16-1027.pdf</t>
+          <t>https://arxiv.org/abs/1611.00354</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:VOx2b1Wkg3QC</t>
+          <t>jnoUuGcAAAAJ:eflP2zaiRacC</t>
         </is>
       </c>
     </row>
@@ -3402,77 +3400,77 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Transliteration</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>IIT Bombay’s English-Indonesian submission at WAT: Integrating neural language models with SMT</t>
+          <t>Substring-based Unsupervised Transliteration with Phonetic and Contextual Knowledge</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>WAT</t>
+          <t>CoNLL</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>Sandhya Singh,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Mitesh Khapra Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W16-4604/</t>
+          <t>https://aclanthology.org/K16-1027.pdf</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>Shared Task</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:wbdj-CoPYUoC</t>
+          <t>jnoUuGcAAAAJ:VOx2b1Wkg3QC</t>
         </is>
       </c>
     </row>
     <row r="74" ht="45" customHeight="1">
       <c r="A74" s="4" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>NLP/Transliteration/Indic/Multilingual</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Brahmi-Net: A transliteration and script conversion system for languages of the Indian subcontinent</t>
+          <t>IIT Bombay’s English-Indonesian submission at WAT: Integrating neural language models with SMT</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>NAACL: System Demonstrations</t>
+          <t>WAT</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Ratish Puduppully,  Pushpak Bhattacharyya</t>
+          <t>Sandhya Singh,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/N15-3017.pdf</t>
+          <t>https://aclanthology.org/W16-4604/</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>Demo</t>
+          <t>Shared Task</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:738O_yMBCRsC</t>
+          <t>jnoUuGcAAAAJ:wbdj-CoPYUoC</t>
         </is>
       </c>
     </row>
@@ -3482,37 +3480,37 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>NLP</t>
+          <t>NLP/Transliteration/Indic/Multilingual</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>SarcasmBot: An open-source sarcasm-generation module for chatbots</t>
+          <t>Brahmi-Net: A transliteration and script conversion system for languages of the Indian subcontinent</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>WISDOM Workshop</t>
+          <t>NAACL: System Demonstrations</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>Aditya Joshi,  Anoop Kunchukuttan,  Pushpak Bhattacharyya,  Mark James Carman</t>
+          <t>Anoop Kunchukuttan,  Ratish Puduppully,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t>https://www.sentic.net/wisdom2015joshi.pdf</t>
+          <t>https://aclanthology.org/N15-3017.pdf</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Demo</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:l7t_Zn2s7bgC</t>
+          <t>jnoUuGcAAAAJ:738O_yMBCRsC</t>
         </is>
       </c>
     </row>
@@ -3522,37 +3520,37 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>NLP/Transliteration</t>
+          <t>NLP</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Data representation methods and use of mined corpora for Indian language transliteration</t>
+          <t>SarcasmBot: An open-source sarcasm-generation module for chatbots</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Proceedings of the Fifth Named Entity Workshop</t>
+          <t>WISDOM Workshop</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Aditya Joshi,  Anoop Kunchukuttan,  Pushpak Bhattacharyya,  Mark James Carman</t>
         </is>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W15-3912.pdf</t>
+          <t>https://www.sentic.net/wisdom2015joshi.pdf</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>Shared Task</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:K3LRdlH-MEoC</t>
+          <t>jnoUuGcAAAAJ:l7t_Zn2s7bgC</t>
         </is>
       </c>
     </row>
@@ -3562,37 +3560,37 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Transliteration</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Augmenting Pivot based SMT with word segmentation</t>
+          <t>Data representation methods and use of mined corpora for Indian language transliteration</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>International Conference on Natural Language Processing (ICON)</t>
+          <t>Proceedings of the Fifth Named Entity Workshop</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>Rohit More,  Anoop Kunchukuttan,  Raj Dabre,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W15-5944.pdf</t>
+          <t>https://aclanthology.org/W15-3912.pdf</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>Short Paper</t>
+          <t>Shared Task</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:vRqMK49ujn8C</t>
+          <t>jnoUuGcAAAAJ:K3LRdlH-MEoC</t>
         </is>
       </c>
     </row>
@@ -3602,12 +3600,12 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>NLP/Grammar-Correction</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Addressing Class Imbalance in Grammatical Error Detection with Evaluation Metric Optimization</t>
+          <t>Augmenting Pivot based SMT with word segmentation</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -3617,22 +3615,22 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Rohit More,  Anoop Kunchukuttan,  Raj Dabre,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W15-5902.pdf</t>
+          <t>https://aclanthology.org/W15-5944.pdf</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Short Paper</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:tS2w5q8j5-wC</t>
+          <t>jnoUuGcAAAAJ:vRqMK49ujn8C</t>
         </is>
       </c>
     </row>
@@ -3642,12 +3640,12 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Grammar-Correction</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Investigating the potential of postordering SMT output to improve translation quality</t>
+          <t>Addressing Class Imbalance in Grammatical Error Detection with Evaluation Metric Optimization</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -3657,22 +3655,22 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Pratik Mehta,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W15-5950.pdf</t>
+          <t>https://aclanthology.org/W15-5902.pdf</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:4fKUyHm3Qg0C</t>
+          <t>jnoUuGcAAAAJ:tS2w5q8j5-wC</t>
         </is>
       </c>
     </row>
@@ -3682,77 +3680,77 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Multilingual</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Translation &amp; Transliteration between Related Languages</t>
+          <t>Investigating the potential of postordering SMT output to improve translation quality</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICON </t>
+          <t>International Conference on Natural Language Processing (ICON)</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Mitesh Khapra</t>
-        </is>
-      </c>
-      <c r="F80" s="1" t="inlineStr">
-        <is>
-          <t>publications/presentations/icon-2015-tutorial-translation-related-lang-slides.pdf</t>
+          <t>Pratik Mehta,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+        </is>
+      </c>
+      <c r="F80" s="10" t="inlineStr">
+        <is>
+          <t>https://aclanthology.org/W15-5950.pdf</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>Tutorial</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:geHnlv5EZngC</t>
+          <t>jnoUuGcAAAAJ:4fKUyHm3Qg0C</t>
         </is>
       </c>
     </row>
     <row r="81" ht="45" customHeight="1">
       <c r="A81" s="4" t="n">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Indic/Multilingual</t>
+          <t>NLP/Translation/Multilingual</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Śata-Anuva̅dak: Tackling Multiway Translation of Indian Languages</t>
+          <t>Translation &amp; Transliteration between Related Languages</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Language Resources and Evaluation Conference</t>
+          <t xml:space="preserve">ICON </t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Abhijit Mishra,  Chatterjee Rajen,  Ritesh Shah,  Pushpak Bhattacharyya</t>
-        </is>
-      </c>
-      <c r="F81" s="10" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Anoop Kunchukuttan,  Mitesh Khapra</t>
+        </is>
+      </c>
+      <c r="F81" s="1" t="inlineStr">
+        <is>
+          <t>publications/presentations/icon-2015-tutorial-translation-related-lang-slides.pdf</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:IjCSPb-OGe4C</t>
+          <t>jnoUuGcAAAAJ:geHnlv5EZngC</t>
         </is>
       </c>
     </row>
@@ -3762,37 +3760,37 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Crowdsourcing</t>
+          <t>NLP/Translation/Indic/Multilingual</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Crowdsourcing translation services</t>
+          <t>Śata-Anuva̅dak: Tackling Multiway Translation of Indian Languages</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
+          <t>Language Resources and Evaluation Conference</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>Anoop Kunchukuttan,  Abhijit Mishra,  Chatterjee Rajen,  Ritesh Shah,  Pushpak Bhattacharyya</t>
+        </is>
+      </c>
+      <c r="F82" s="10" t="inlineStr">
+        <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="E82" s="4" t="inlineStr">
-        <is>
-          <t>Anoop Kunchukuttan,  Shourya Roy,  Mitesh Khapra,  Nicola Cancedda,  Pushpak Bhattacharyya</t>
-        </is>
-      </c>
-      <c r="F82" s="10" t="inlineStr">
-        <is>
-          <t>https://patents.google.com/patent/US20140058718A1/en</t>
-        </is>
-      </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>Patent</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:W7OEmFMy1HYC</t>
+          <t>jnoUuGcAAAAJ:IjCSPb-OGe4C</t>
         </is>
       </c>
     </row>
@@ -3802,37 +3800,37 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Translation/Crowdsourcing</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>The IIT Bombay Hindi⇔ English Translation System at WMT 2014</t>
+          <t>Crowdsourcing translation services</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>ICON Shared Task</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>Piyush Dungarwal,  Rajen Chatterjee,  Abhijit Mishra,  Anoop Kunchukuttan,  Ritesh Shah,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Shourya Roy,  Mitesh Khapra,  Nicola Cancedda,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W14-3308.pdf</t>
+          <t>https://patents.google.com/patent/US20140058718A1/en</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>Shared Task</t>
+          <t>Patent</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:SP6oXDckpogC</t>
+          <t>jnoUuGcAAAAJ:W7OEmFMy1HYC</t>
         </is>
       </c>
     </row>
@@ -3842,37 +3840,37 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>NLP/Transliteration/Crowdsourcing</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>When Transliteration Met Crowdsourcing : An Empirical Study of Transliteration via Crowdsourcing using Efficient, Non-redundant and Fair Quality Control</t>
+          <t>The IIT Bombay Hindi⇔ English Translation System at WMT 2014</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Language and Resources and Evaluation Conference</t>
+          <t>ICON Shared Task</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Mitesh Khapra,  Ananthakrishnan Ramanathan,  Anoop Kunchukuttan,  Karthik Visweswariah,  Pushpak Bhattacharyya</t>
+          <t>Piyush Dungarwal,  Rajen Chatterjee,  Abhijit Mishra,  Anoop Kunchukuttan,  Ritesh Shah,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t>https://www.cse.iitb.ac.in/~anoopk/publications/lrec2014_transliteration_crowdsourcing.pdf</t>
+          <t>https://aclanthology.org/W14-3308.pdf</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Shared Task</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:Y0pCki6q_DkC</t>
+          <t>jnoUuGcAAAAJ:SP6oXDckpogC</t>
         </is>
       </c>
     </row>
@@ -3882,37 +3880,37 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Transliteration/Crowdsourcing</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>The IIT Bombay SMT System for ICON 2014 Tools Contest</t>
+          <t>When Transliteration Met Crowdsourcing : An Empirical Study of Transliteration via Crowdsourcing using Efficient, Non-redundant and Fair Quality Control</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>NLP Tools Contest at ICON 2014</t>
+          <t>Language and Resources and Evaluation Conference</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Ratish Pudupully,  Rajen Chatterjee,  Abhijit Mishra,  Pushpak Bhattacharyya</t>
+          <t>Mitesh Khapra,  Ananthakrishnan Ramanathan,  Anoop Kunchukuttan,  Karthik Visweswariah,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t>https://www.cse.iitb.ac.in/~anoopk/publications/icon_2014_iitbsys.pdf</t>
+          <t>https://www.cse.iitb.ac.in/~anoopk/publications/lrec2014_transliteration_crowdsourcing.pdf</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>Shared Task</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:u9iWguZQMMsC</t>
+          <t>jnoUuGcAAAAJ:Y0pCki6q_DkC</t>
         </is>
       </c>
     </row>
@@ -3922,27 +3920,27 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>NLP/Grammar-Correction</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Tuning a grammar correction system for increased precision</t>
+          <t>The IIT Bombay SMT System for ICON 2014 Tools Contest</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Proceedings of the Eighteenth Conference on Computational Natural Language Learning: Shared Task</t>
+          <t>NLP Tools Contest at ICON 2014</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Sriram Chaudhury,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Ratish Pudupully,  Rajen Chatterjee,  Abhijit Mishra,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W14-1708.pdf</t>
+          <t>https://www.cse.iitb.ac.in/~anoopk/publications/icon_2014_iitbsys.pdf</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr">
@@ -3952,7 +3950,7 @@
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:UxriW0iASnsC</t>
+          <t>jnoUuGcAAAAJ:u9iWguZQMMsC</t>
         </is>
       </c>
     </row>
@@ -3962,37 +3960,37 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Grammar-Correction</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Supertag Based Pre-ordering in Machine Translation</t>
+          <t>Tuning a grammar correction system for increased precision</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>International Conference on Natural Language Processing</t>
+          <t>Proceedings of the Eighteenth Conference on Computational Natural Language Learning: Shared Task</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>Rajen Chatterjee,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Sriram Chaudhury,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W14-5105.pdf</t>
+          <t>https://aclanthology.org/W14-1708.pdf</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Shared Task</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:p2g8aNsByqUC</t>
+          <t>jnoUuGcAAAAJ:UxriW0iASnsC</t>
         </is>
       </c>
     </row>
@@ -4007,32 +4005,32 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Machine Learning For Machine Translation</t>
+          <t>Supertag Based Pre-ordering in Machine Translation</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICON </t>
+          <t>International Conference on Natural Language Processing</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>Pushpak Bhattacharyya,  Anoop Kunchukuttan,  Piyush Dungarwal,  Shubham Gautam</t>
+          <t>Rajen Chatterjee,  Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t>publications/presentations/icon_2013_smt_tutorial_slides.pdf</t>
+          <t>https://aclanthology.org/W14-5105.pdf</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>Tutorial</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:LPZeul_q3PIC</t>
+          <t>jnoUuGcAAAAJ:p2g8aNsByqUC</t>
         </is>
       </c>
     </row>
@@ -4047,72 +4045,72 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Boosting Phrase-based SMT with Unsupervised Morph-Analysis and Transliteration Mining</t>
+          <t>Machine Learning For Machine Translation</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>NLP Tools Contest: ICON 2014</t>
+          <t xml:space="preserve">ICON </t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Ratish Puduppully,  Rajen Chatterjee,  Abhijit Mishra,  Pushpak Bhattacharyya</t>
+          <t>Pushpak Bhattacharyya,  Anoop Kunchukuttan,  Piyush Dungarwal,  Shubham Gautam</t>
         </is>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>publications/presentations/icon_2013_smt_tutorial_slides.pdf</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:XiSMed-E-HIC</t>
+          <t>jnoUuGcAAAAJ:LPZeul_q3PIC</t>
         </is>
       </c>
     </row>
     <row r="90" ht="60" customHeight="1">
       <c r="A90" s="4" t="n">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>NLP/Grammar-Correction</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>IITB System for CoNLL 2013 Shared Task: A Hybrid Approach to Grammatical Error Correction</t>
+          <t>Boosting Phrase-based SMT with Unsupervised Morph-Analysis and Transliteration Mining</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Proceedings of the Seventeenth Conference on Computational Natural Language Learning</t>
+          <t>NLP Tools Contest: ICON 2014</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Ritesh Shah,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Ratish Puduppully,  Rajen Chatterjee,  Abhijit Mishra,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W13-3611.pdf</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>Shared Task</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:UeHWp8X0CEIC</t>
+          <t>jnoUuGcAAAAJ:XiSMed-E-HIC</t>
         </is>
       </c>
     </row>
@@ -4122,43 +4120,43 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation/Crowdsourcing</t>
+          <t>NLP/Grammar-Correction</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>TransDoop: A Map-Reduce based Crowdsourced Translation for Complex Domain</t>
+          <t>IITB System for CoNLL 2013 Shared Task: A Hybrid Approach to Grammatical Error Correction</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>Proceedings of the Association of Computational Linguistics (demo)</t>
+          <t>Proceedings of the Seventeenth Conference on Computational Natural Language Learning</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Rajen Chatterjee,  Shourya Roy,  Abhijit Mishra,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Ritesh Shah,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/P13-4030.pdf</t>
+          <t>https://aclanthology.org/W13-3611.pdf</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>Demo</t>
+          <t>Shared Task</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:qjMakFHDy7sC</t>
+          <t>jnoUuGcAAAAJ:UeHWp8X0CEIC</t>
         </is>
       </c>
     </row>
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="4" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
@@ -4167,32 +4165,32 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Experiences in resource generation for machine translation through crowdsourcing</t>
+          <t>TransDoop: A Map-Reduce based Crowdsourced Translation for Complex Domain</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>LREC</t>
+          <t>Proceedings of the Association of Computational Linguistics (demo)</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Shourya Roy,  Pratik Patel,  Kushal Ladha,  Somya Gupta,  Mitesh Khapra,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Rajen Chatterjee,  Shourya Roy,  Abhijit Mishra,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=8c2b058d70ca908ff348b6b5c6b5cdd892a76cc2</t>
+          <t>https://aclanthology.org/P13-4030.pdf</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Demo</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:7T2F9Uy0os0C</t>
+          <t>jnoUuGcAAAAJ:qjMakFHDy7sC</t>
         </is>
       </c>
     </row>
@@ -4202,37 +4200,37 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/Translation/Crowdsourcing</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Partially modelling word reordering as a sequence labelling problem</t>
+          <t>Experiences in resource generation for machine translation through crowdsourcing</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Workshop on Reordering for Statistical Machine Translation</t>
+          <t>LREC</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Shourya Roy,  Pratik Patel,  Kushal Ladha,  Somya Gupta,  Mitesh Khapra,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/W12-5906.pdf</t>
+          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=8c2b058d70ca908ff348b6b5c6b5cdd892a76cc2</t>
         </is>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>Shared Task</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:2osOgNQ5qMEC</t>
+          <t>jnoUuGcAAAAJ:7T2F9Uy0os0C</t>
         </is>
       </c>
     </row>
@@ -4242,37 +4240,37 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>NLP/MWE</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Multiword Expressions in the CLIA Project</t>
+          <t>Partially modelling word reordering as a sequence labelling problem</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>Vishwabharat</t>
+          <t>Workshop on Reordering for Statistical Machine Translation</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Munish Minia,  Pushpak Bhattacharyya</t>
+          <t>Anoop Kunchukuttan,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t>/files/papers/clia_mwe_vishwabharat_2012.pdf</t>
+          <t>https://aclanthology.org/W12-5906.pdf</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>Shared Task</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:8AbLer7MMksC</t>
+          <t>jnoUuGcAAAAJ:2osOgNQ5qMEC</t>
         </is>
       </c>
     </row>
@@ -4282,27 +4280,27 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>NLP/Translation</t>
+          <t>NLP/MWE</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>The Reordering Problem in Statistical Machine Translation</t>
+          <t>Multiword Expressions in the CLIA Project</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Vishwabharat</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan</t>
+          <t>Anoop Kunchukuttan,  Munish Minia,  Pushpak Bhattacharyya</t>
         </is>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>/files/papers/clia_mwe_vishwabharat_2012.pdf</t>
         </is>
       </c>
       <c r="G95" s="4" t="inlineStr">
@@ -4312,53 +4310,53 @@
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:OU6Ihb5iCvQC</t>
+          <t>jnoUuGcAAAAJ:8AbLer7MMksC</t>
         </is>
       </c>
     </row>
     <row r="96" ht="45" customHeight="1">
       <c r="A96" s="4" t="n">
-        <v>2008</v>
+        <v>2012</v>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>NLP/MWE</t>
+          <t>NLP/Translation</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>A system for compound noun multiword expression extraction for hindi</t>
+          <t>The Reordering Problem in Statistical Machine Translation</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>ICON</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan,  Om Prakash Damani</t>
+          <t>Anoop Kunchukuttan</t>
         </is>
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=b3322b5d48b950cbdebb1cae41509486acbed27a</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>Full Paper</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="H96" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:u5HHmVD_uO8C</t>
+          <t>jnoUuGcAAAAJ:OU6Ihb5iCvQC</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
@@ -4367,77 +4365,117 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Multiword Expression Recognition</t>
+          <t>A system for compound noun multiword expression extraction for hindi</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ICON</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>Anoop Kunchukuttan</t>
+          <t>Anoop Kunchukuttan,  Om Prakash Damani</t>
         </is>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=3e3fd0173dcb28aa1a11d5342da527a835235ae4</t>
+          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=b3322b5d48b950cbdebb1cae41509486acbed27a</t>
         </is>
       </c>
       <c r="G97" s="4" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Full Paper</t>
         </is>
       </c>
       <c r="H97" s="4" t="inlineStr">
         <is>
-          <t>jnoUuGcAAAAJ:9yKSN-GCB0IC</t>
+          <t>jnoUuGcAAAAJ:u5HHmVD_uO8C</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>NLP/MWE</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>Multiword Expression Recognition</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>Anoop Kunchukuttan</t>
+        </is>
+      </c>
+      <c r="F98" s="10" t="inlineStr">
+        <is>
+          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=3e3fd0173dcb28aa1a11d5342da527a835235ae4</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>jnoUuGcAAAAJ:9yKSN-GCB0IC</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="n">
         <v>2006</v>
       </c>
-      <c r="B98" s="4" t="inlineStr">
+      <c r="B99" s="4" t="inlineStr">
         <is>
           <t>Misc</t>
         </is>
       </c>
-      <c r="C98" s="4" t="inlineStr">
+      <c r="C99" s="4" t="inlineStr">
         <is>
           <t>Evaluation of Information Retrieval Systems</t>
         </is>
       </c>
-      <c r="D98" s="4" t="inlineStr">
+      <c r="D99" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="E98" s="4" t="inlineStr">
+      <c r="E99" s="4" t="inlineStr">
         <is>
           <t>Anoop Kunchukuttan</t>
         </is>
       </c>
-      <c r="F98" s="10" t="inlineStr">
+      <c r="F99" s="10" t="inlineStr">
         <is>
           <t>http://www.kramirez.net/RI/Material/Internet/Evaluacion/seminar06_presentation.pdf</t>
         </is>
       </c>
-      <c r="G98" s="4" t="inlineStr">
+      <c r="G99" s="4" t="inlineStr">
         <is>
           <t>Survey</t>
         </is>
       </c>
-      <c r="H98" s="4" t="inlineStr">
+      <c r="H99" s="4" t="inlineStr">
         <is>
           <t>jnoUuGcAAAAJ:u-x6o8ySG0sC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J98"/>
+  <autoFilter ref="A1:J99"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>

</xml_diff>